<commit_message>
feat(presupuestos): incorporar 2 escaleras de gato opcionales con crinolina en acero inoxidable para voladizo y cubierta a P-2026-0044
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
+++ b/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,7 +32,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000F172A"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -43,11 +43,53 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E1B4B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00EF4444"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -55,38 +97,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="9.5"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00B91C1C"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="001E1B4B"/>
-      <sz val="15"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00EF4444"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +127,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEF2F2"/>
         <bgColor rgb="00FEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -164,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -208,27 +238,57 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -236,14 +296,13 @@
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -609,11 +668,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -690,7 +749,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado especial anticorrosión marina Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones inoxidables bimetálicas A2 con arandela EPDM | Sellado continuo de butilo</t>
+          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado especial anticorrosión marina Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones bimetálicas inox A2 + EPDM | Opcionales: 2 escalas de gato con crinolina en ACERO INOXIDABLE (UNE-EN ISO 14122-4)</t>
         </is>
       </c>
     </row>
@@ -845,7 +904,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>VALORACIÓN ECONÓMICA DE PARTIDAS</t>
+          <t>VALORACIÓN ECONÓMICA DE PARTIDAS BASE</t>
         </is>
       </c>
     </row>
@@ -1077,89 +1136,250 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="E27" s="21" t="inlineStr">
+        <is>
+          <t>Subtotal Base Imponible (Obra Base):</t>
+        </is>
+      </c>
+      <c r="F27" s="22">
+        <f>SUM(F20:F26)</f>
+        <v/>
+      </c>
+    </row>
     <row r="28">
-      <c r="E28" s="21" t="inlineStr">
-        <is>
-          <t>Base Imponible:</t>
-        </is>
-      </c>
-      <c r="F28" s="22">
-        <f>SUM(F20:F26)</f>
+      <c r="E28" s="23" t="inlineStr">
+        <is>
+          <t>I.V.A. (21%) Obra Base:</t>
+        </is>
+      </c>
+      <c r="F28" s="24">
+        <f>F27*0.21</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>I.V.A. (21%):</t>
-        </is>
-      </c>
-      <c r="F29" s="22">
-        <f>F28*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>TOTAL PRESUPUESTO:</t>
-        </is>
-      </c>
-      <c r="F30" s="24">
-        <f>F28+F29</f>
-        <v/>
+      <c r="E29" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL OBRA BASE (IVA incl.):</t>
+        </is>
+      </c>
+      <c r="F29" s="26">
+        <f>F27+F28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>PARTIDAS OPCIONALES INDEPENDIENTES (ACCESOS DE SEGURIDAD EN ACERO INOXIDABLE)</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>Partida</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Concepto y Descripción Técnica</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
+        <is>
+          <t>Precio Unitario (€)</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="inlineStr">
+        <is>
+          <t>Importe (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>OPC-01</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>OPCIONAL 1: Escalera de gato con protección dorsal en acero inoxidable para acceso a voladizo (H ≈ 4,20 m)
+Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso seguro desde cota suelo a voladizo (altura aprox. 4,20 m, desarrollo total 5,30 m con desembarco). Incluye montantes verticales de pletina/tubo inox, peldaños antideslizantes estriados de seguridad, jaula de protección dorsal (crinolina) aros y tirantes longitudinales en pletina inox a partir de 2,20 m, desembarco superior ensanchado con barandillas de salida de 1.100 mm, compuerta batiente de gravedad/muelle con cierre automático, placa de condena inferior anti-intrusión con candado en acero inoxidable para control de acceso aeroportuario Aena, y anclajes químicos de alta resistencia en acero inox A4.</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>3850</v>
+      </c>
+      <c r="F33" s="20">
+        <f>D33*E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>OPC-02</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>OPCIONAL 2: Escalera de gato con protección dorsal en acero inoxidable para acceso a cubierta (H ≈ 6,80 m)
+Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso técnico y de mantenimiento a la cubierta principal del edificio (altura aprox. 6,80 m, desarrollo total 7,90 m con desembarco). Incluye montantes de acero inox, peldaños antideslizantes mecanizados, jaula dorsal continua (crinolina) en acero inox a partir de 2,50 m de altura, desembarco superior protegido con barandillas de 1.100 mm y rodapié, puerta batiente de salida con resorte de cierre automático de seguridad, portón inferior abatible de bloqueo anti-intrusión con cerradura/candado de seguridad en acero inoxidable, y fijaciones estructurales en acero inoxidable A4.</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <v>5950</v>
+      </c>
+      <c r="F34" s="20">
+        <f>D34*E34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>Subtotal Opcionales (Base Imp.):</t>
+        </is>
+      </c>
+      <c r="F35" s="30">
+        <f>SUM(F33:F34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>I.V.A. (21%) Opcionales:</t>
+        </is>
+      </c>
+      <c r="F36" s="24">
+        <f>F35*0.21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" s="31" t="inlineStr">
+        <is>
+          <t>TOTAL OPCIONALES (IVA incl.):</t>
+        </is>
+      </c>
+      <c r="F37" s="32">
+        <f>F35+F36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL BASE IMPONIBLE CONJUNTA:</t>
+        </is>
+      </c>
+      <c r="F39" s="34">
+        <f>F27+F35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" s="35" t="inlineStr">
+        <is>
+          <t>I.V.A. (21%) Conjunto:</t>
+        </is>
+      </c>
+      <c r="F40" s="36">
+        <f>F39*0.21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" s="37" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL CONTRATO (IVA incl.):</t>
+        </is>
+      </c>
+      <c r="F41" s="38">
+        <f>F39+F40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>CONDICIONES COMERCIALES Y DE EJECUCIÓN</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>• Forma de pago:</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>40% a la formalización (106.588,90 € con IVA), 30% a la recepción en obra de materiales (79.941,68 € con IVA) y 30% a la recepción final conforme (79.941,67 € con IVA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>40% a la formalización (106.588,90 € base), 30% al acopio e inicio montaje (79.941,68 €) y 30% a la recepción final (79.941,67 €). Las partidas opcionales se facturan según aprobación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>• Plazo de ejecución:</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>5 a 7 semanas laborables desde recepción y acopio de paneles en Menorca</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>5 a 7 semanas laborables desde recepción de paneles en Menorca</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>• Garantías:</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>10 años en recubrimiento Granite® HDX55 contra corrosión marina y perforación; 5 años en estanqueidad de cubierta; 2 años en montaje y remates</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>10 años en recubrimiento Granite® HDX55 y en acero inoxidable; 5 años en estanqueidad; 2 años en montaje y mecanismos</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>• Validez de oferta:</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>30 días naturales desde la fecha de emisión</t>
         </is>
@@ -1176,28 +1396,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="39" t="inlineStr">
         <is>
           <t>HAM ESTRUCTURAS METÁLICAS - ESCANDALLO DE COMPRA Y COSTES DIRECTOS INTERNOS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>CONFIDENCIAL: USO INTERNO EXCLUSIVO · COSTES DIRECTOS Y ANÁLISIS DE RENTABILIDAD</t>
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>CONFIDENCIAL: USO INTERNO EXCLUSIVO · COSTES DIRECTOS Y ANÁLISIS DE RENTABILIDAD (OBRA BASE + OPCIONALES)</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1434,12 @@
           <t>Coste compra Panel Sándwich HDX55 2 caras (40 mm PIR):</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="36" t="n">
         <v>36</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>€/m² (acopio en fábrica Península)</t>
+          <t>€/m² (acopio fábrica Península)</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1449,7 @@
           <t>Coste compra Panel/Chapa HDX55 Voladizos 2 caras:</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="36" t="n">
         <v>34</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1244,7 +1464,7 @@
           <t>Tarifa interna mano de obra oficial montaje:</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="36" t="n">
         <v>28</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1261,32 +1481,32 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="41" t="inlineStr">
         <is>
           <t>Capítulo</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="42" t="inlineStr">
         <is>
           <t>Concepto de Coste Interno</t>
         </is>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="C10" s="41" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D10" s="27" t="inlineStr">
+      <c r="D10" s="41" t="inlineStr">
         <is>
           <t>Medición</t>
         </is>
       </c>
-      <c r="E10" s="27" t="inlineStr">
+      <c r="E10" s="41" t="inlineStr">
         <is>
           <t>Coste Unit. HAM (€)</t>
         </is>
       </c>
-      <c r="F10" s="27" t="inlineStr">
+      <c r="F10" s="41" t="inlineStr">
         <is>
           <t>Coste Total HAM (€)</t>
         </is>
@@ -1300,7 +1520,7 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Panel sándwich 40 mm PIR con acabado HDX55 en 2 caras para cubiertas (1.371 m² + 5% solapes/mermas)</t>
+          <t>Panel sándwich 40 mm PIR con acabado HDX55 en 2 caras cubiertas (1.371 m² + 5% solapes/mermas)</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
@@ -1328,7 +1548,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Panel / chapa autoportante acabado HDX55 en 2 caras para voladizos (533 m² + 5% mermas)</t>
+          <t>Panel / chapa grecada acabado HDX55 en 2 caras para voladizos (533 m² + 5% mermas)</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
@@ -1432,25 +1652,24 @@
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>MO-01</t>
+          <t>MAT-06</t>
         </is>
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>Mano de obra especializada desmontaje y montaje HAM (cuadrilla de 4 oficiales ~800 h)</t>
+          <t>Materiales y perfiles en ACERO INOXIDABLE (AISI 304/316) para 2 escaleras con crinolina y cancelas</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>horas</t>
+          <t>lote</t>
         </is>
       </c>
       <c r="D16" s="19" t="n">
-        <v>800</v>
-      </c>
-      <c r="E16" s="20">
-        <f>B7</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>3700</v>
       </c>
       <c r="F16" s="20">
         <f>D16*E16</f>
@@ -1460,24 +1679,25 @@
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>LOG-01</t>
+          <t>MO-01</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>Fletes marítimos Península-Menorca para trailers especiales con paneles de gran formato</t>
+          <t>Mano de obra especializada montaje HAM obra base (cuadrilla de 4 oficiales ~800 h)</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>lote</t>
+          <t>horas</t>
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="20" t="n">
-        <v>5200</v>
+        <v>800</v>
+      </c>
+      <c r="E17" s="20">
+        <f>B7</f>
+        <v/>
       </c>
       <c r="F17" s="20">
         <f>D17*E17</f>
@@ -1487,24 +1707,25 @@
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>LOG-02</t>
+          <t>MO-02</t>
         </is>
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>Camión grúa pluma autopropulsada para descarga e izado distribuido sobre pórticos</t>
+          <t>Mano de obra montaje e instalación de 2 escaleras inox con crinolina (~60 h taller y montaje)</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>lote</t>
+          <t>horas</t>
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="20" t="n">
-        <v>4600</v>
+        <v>60</v>
+      </c>
+      <c r="E18" s="20">
+        <f>B7</f>
+        <v/>
       </c>
       <c r="F18" s="20">
         <f>D18*E18</f>
@@ -1514,12 +1735,12 @@
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>LOG-03</t>
+          <t>LOG-01</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Alquiler de 2 plataformas elevadoras móviles de personal (PEMP) articuladas durante montaje</t>
+          <t>Fletes marítimos Península-Menorca para transporte de trailers especiales con paneles de gran formato</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
@@ -1531,7 +1752,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="20" t="n">
-        <v>3400</v>
+        <v>5200</v>
       </c>
       <c r="F19" s="20">
         <f>D19*E19</f>
@@ -1541,12 +1762,12 @@
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>PRL-01</t>
+          <t>LOG-02</t>
         </is>
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>Protecciones colectivas: redes anticaídas bajo faldones UNE-EN 1263-1 y líneas de vida EN 795</t>
+          <t>Camión grúa pluma autopropulsada para descarga e izado distribuido sobre pórticos en aeropuerto</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
@@ -1558,7 +1779,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>3800</v>
+        <v>4600</v>
       </c>
       <c r="F20" s="20">
         <f>D20*E20</f>
@@ -1568,12 +1789,12 @@
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>PRL-02</t>
+          <t>LOG-03</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>Canon de vertedero insular y tasas de centro de reciclaje autorizado de Menorca</t>
+          <t>Alquiler de 2 plataformas elevadoras móviles de personal (PEMP) articuladas durante montaje</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -1585,7 +1806,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="20" t="n">
-        <v>1800</v>
+        <v>3400</v>
       </c>
       <c r="F21" s="20">
         <f>D21*E21</f>
@@ -1593,102 +1814,168 @@
       </c>
     </row>
     <row r="22">
-      <c r="E22" s="29" t="inlineStr">
-        <is>
-          <t>COSTE DIRECTO TOTAL (CDT HAM):</t>
-        </is>
-      </c>
-      <c r="F22" s="30">
-        <f>SUM(F11:F21)</f>
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>PRL-01</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Protecciones colectivas: redes anticaídas bajo faldones UNE-EN 1263-1 y líneas de vida EN 795</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>3800</v>
+      </c>
+      <c r="F22" s="20">
+        <f>D22*E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>PRL-02</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Canon de vertedero insular y tasas de centro de reciclaje autorizado de Menorca</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F23" s="20">
+        <f>D23*E23</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="E24" s="43" t="inlineStr">
+        <is>
+          <t>COSTE DIRECTO TOTAL GLOBAL (CDT HAM):</t>
+        </is>
+      </c>
+      <c r="F24" s="44">
+        <f>SUM(F11:F23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>CUADRO DE RENTABILIDAD Y BENEFICIO COMERCIAL</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="31" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="45" t="inlineStr">
         <is>
           <t>Concepto Económico</t>
         </is>
       </c>
-      <c r="B25" s="31" t="inlineStr">
-        <is>
-          <t>Importe (€)</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>% sobre Venta</t>
-        </is>
-      </c>
-      <c r="D25" s="31" t="inlineStr">
-        <is>
-          <t>Observaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="32" t="inlineStr">
-        <is>
-          <t>Precio de Venta al Cliente (Base Imponible):</t>
-        </is>
-      </c>
-      <c r="B26" s="33">
-        <f>'Presupuesto Cliente'!F28</f>
-        <v/>
-      </c>
-      <c r="C26" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>PVP ofertado a UG21 / Aena</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="32" t="inlineStr">
-        <is>
-          <t>Coste Directo Total de Ejecución HAM:</t>
-        </is>
-      </c>
-      <c r="B27" s="33">
-        <f>F22</f>
-        <v/>
-      </c>
-      <c r="C27" s="34">
-        <f>B27/B26</f>
-        <v/>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Materiales (67%) + MO (18%) + Logística y Medios (15%)</t>
+      <c r="B27" s="45" t="inlineStr">
+        <is>
+          <t>Obra Base (€)</t>
+        </is>
+      </c>
+      <c r="C27" s="45" t="inlineStr">
+        <is>
+          <t>Opcionales Inox (€)</t>
+        </is>
+      </c>
+      <c r="D27" s="45" t="inlineStr">
+        <is>
+          <t>Total Global (€)</t>
+        </is>
+      </c>
+      <c r="E27" s="45" t="inlineStr">
+        <is>
+          <t>% Margen Global</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="35" t="inlineStr">
+      <c r="A28" s="46" t="inlineStr">
+        <is>
+          <t>Precio de Venta al Cliente (Base Imp.):</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="n">
+        <v>220225</v>
+      </c>
+      <c r="C28" s="47" t="n">
+        <v>9800</v>
+      </c>
+      <c r="D28" s="47">
+        <f>B28+C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="48" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="46" t="inlineStr">
+        <is>
+          <t>Coste Directo Total HAM:</t>
+        </is>
+      </c>
+      <c r="B29" s="47" t="n">
+        <v>125530</v>
+      </c>
+      <c r="C29" s="47" t="n">
+        <v>5380</v>
+      </c>
+      <c r="D29" s="47">
+        <f>B29+C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="48">
+        <f>D29/D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
         <is>
           <t>Margen Bruto de Explotación HAM:</t>
         </is>
       </c>
-      <c r="B28" s="36">
-        <f>B26-B27</f>
-        <v/>
-      </c>
-      <c r="C28" s="37">
-        <f>B28/B26</f>
-        <v/>
-      </c>
-      <c r="D28" s="38" t="inlineStr">
-        <is>
-          <t>Beneficio bruto de explotación de la actuación</t>
-        </is>
+      <c r="B30" s="50">
+        <f>B28-B29</f>
+        <v/>
+      </c>
+      <c r="C30" s="50">
+        <f>C28-C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="50">
+        <f>D28-D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="51">
+        <f>D30/D28</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(presupuestos): subir un 30% escaleras inox y anadir linea de vida LuxTop 18.000 EUR como opcional a P-2026-0044
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
+++ b/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
@@ -71,7 +71,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001E3A8A"/>
-      <sz val="12"/>
+      <sz val="11.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -749,7 +749,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado especial anticorrosión marina Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones bimetálicas inox A2 + EPDM | Opcionales: 2 escalas de gato con crinolina en ACERO INOXIDABLE (UNE-EN ISO 14122-4)</t>
+          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado especial anticorrosión marina Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones bimetálicas inox A2 + EPDM | Opcionales: 2 escalas de gato inox con crinolina (+30%) + Línea de vida permanente LuxTop® (18.000 €)</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>PARTIDAS OPCIONALES INDEPENDIENTES (ACCESOS DE SEGURIDAD EN ACERO INOXIDABLE)</t>
+          <t>PARTIDAS OPCIONALES INDEPENDIENTES (ACCESOS EN ACERO INOXIDABLE Y LÍNEA DE VIDA LUXTOP)</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       <c r="B33" s="18" t="inlineStr">
         <is>
           <t>OPCIONAL 1: Escalera de gato con protección dorsal en acero inoxidable para acceso a voladizo (H ≈ 4,20 m)
-Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso seguro desde cota suelo a voladizo (altura aprox. 4,20 m, desarrollo total 5,30 m con desembarco). Incluye montantes verticales de pletina/tubo inox, peldaños antideslizantes estriados de seguridad, jaula de protección dorsal (crinolina) aros y tirantes longitudinales en pletina inox a partir de 2,20 m, desembarco superior ensanchado con barandillas de salida de 1.100 mm, compuerta batiente de gravedad/muelle con cierre automático, placa de condena inferior anti-intrusión con candado en acero inoxidable para control de acceso aeroportuario Aena, y anclajes químicos de alta resistencia en acero inox A4.</t>
+Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso seguro desde cota suelo a voladizo (altura aprox. 4,20 m, desarrollo total 5,30 m con desembarco). Incluye montantes verticales de pletina/tubo inox, peldaños antideslizantes estriados de seguridad, jaula de protección dorsal (crinolina) con aros y tirantes longitudinales en pletina inox a partir de 2,20 m, desembarco superior ensanchado con barandillas de salida de 1.100 mm, compuerta batiente de gravedad/muelle con cierre automático, placa de condena inferior anti-intrusión con candado en acero inoxidable para control de acceso aeroportuario AENA, y anclajes químicos estructurales en acero inox A4.</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
@@ -1229,7 +1229,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>3850</v>
+        <v>5005</v>
       </c>
       <c r="F33" s="20">
         <f>D33*E33</f>
@@ -1257,7 +1257,7 @@
         <v>1</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>5950</v>
+        <v>7735</v>
       </c>
       <c r="F34" s="20">
         <f>D34*E34</f>
@@ -1265,121 +1265,149 @@
       </c>
     </row>
     <row r="35">
-      <c r="E35" s="29" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>OPC-03</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>OPCIONAL 3: Línea de vida permanente homologada marca LuxTop® sobre cubierta
+Suministro, replanteo, montaje y certificación oficial de sistema permanente de línea de vida horizontal continua de cable de acero inoxidable AISI 316 (Ø 8 mm) marca LUXTOP®, conforme a las normas UNE-EN 795:2012 Tipo C y CEN/TS 16415 (homologada para trabajo y rescate de hasta 4 operarios simultáneos). Instalación sobre cubierta de panel sándwich mediante postes terminales e intermedios con absorbedor de impacto dinámico patentado LuxTop®, bases de fijación estancas sobreelevadas con juntas de EPDM (evitando cualquier riesgo de filtración o puente térmico), tensor de cable con testigo micrométrico de tensión, pieza curva/esquina si procede, carros deslizadores pasantes transfronterizos sin necesidad de desconexión manual, placa de marcado identificativa CE, ensayos de tracción en obra y dossier de legalización con certificado visado.</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F35" s="20">
+        <f>D35*E35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" s="29" t="inlineStr">
         <is>
           <t>Subtotal Opcionales (Base Imp.):</t>
         </is>
       </c>
-      <c r="F35" s="30">
-        <f>SUM(F33:F34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="E36" s="23" t="inlineStr">
+      <c r="F36" s="30">
+        <f>SUM(F33:F35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" s="23" t="inlineStr">
         <is>
           <t>I.V.A. (21%) Opcionales:</t>
         </is>
       </c>
-      <c r="F36" s="24">
-        <f>F35*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="E37" s="31" t="inlineStr">
+      <c r="F37" s="24">
+        <f>F36*0.21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" s="31" t="inlineStr">
         <is>
           <t>TOTAL OPCIONALES (IVA incl.):</t>
         </is>
       </c>
-      <c r="F37" s="32">
-        <f>F35+F36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="E39" s="33" t="inlineStr">
+      <c r="F38" s="32">
+        <f>F36+F37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" s="33" t="inlineStr">
         <is>
           <t>TOTAL BASE IMPONIBLE CONJUNTA:</t>
         </is>
       </c>
-      <c r="F39" s="34">
-        <f>F27+F35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="E40" s="35" t="inlineStr">
+      <c r="F40" s="34">
+        <f>F27+F36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" s="35" t="inlineStr">
         <is>
           <t>I.V.A. (21%) Conjunto:</t>
         </is>
       </c>
-      <c r="F40" s="36">
-        <f>F39*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="E41" s="37" t="inlineStr">
+      <c r="F41" s="36">
+        <f>F40*0.21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="E42" s="37" t="inlineStr">
         <is>
           <t>TOTAL GENERAL CONTRATO (IVA incl.):</t>
         </is>
       </c>
-      <c r="F41" s="38">
-        <f>F39+F40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>CONDICIONES COMERCIALES Y DE EJECUCIÓN</t>
-        </is>
+      <c r="F42" s="38">
+        <f>F40+F41</f>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>• Forma de pago:</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>40% a la formalización (106.588,90 € base), 30% al acopio e inicio montaje (79.941,68 €) y 30% a la recepción final (79.941,67 €). Las partidas opcionales se facturan según aprobación.</t>
+          <t>CONDICIONES COMERCIALES Y DE EJECUCIÓN</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>• Plazo de ejecución:</t>
+          <t>• Forma de pago:</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>5 a 7 semanas laborables desde recepción de paneles en Menorca</t>
+          <t>40% a la formalización (106.588,90 € base), 30% al acopio e inicio montaje (79.941,68 €) y 30% a la recepción final (79.941,67 €). Las partidas opcionales se facturan según aprobación.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>• Garantías:</t>
+          <t>• Plazo de ejecución:</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>10 años en recubrimiento Granite® HDX55 y en acero inoxidable; 5 años en estanqueidad; 2 años en montaje y mecanismos</t>
+          <t>5 a 7 semanas laborables desde recepción de paneles en Menorca</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
+          <t>• Garantías:</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>10 años en recubrimiento Granite® HDX55, en acero inoxidable y en sistema LuxTop®; 5 años en estanqueidad; 2 años en montaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
           <t>• Validez de oferta:</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>30 días naturales desde la fecha de emisión</t>
         </is>
@@ -1396,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1417,7 +1445,7 @@
     <row r="2">
       <c r="A2" s="40" t="inlineStr">
         <is>
-          <t>CONFIDENCIAL: USO INTERNO EXCLUSIVO · COSTES DIRECTOS Y ANÁLISIS DE RENTABILIDAD (OBRA BASE + OPCIONALES)</t>
+          <t>CONFIDENCIAL: USO INTERNO EXCLUSIVO · OBRA BASE + ESCALERAS INOX (+30%) + LÍNEA LUXTOP</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1604,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Tornillería bimetálica inox A2 con arandelas EPDM, puentes y masilla hidro-expansiva de butilo</t>
+          <t>Tornillería bimetálica inox A2 con arandelas EPDM, accesorios fijación y masilla de butilo</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
@@ -1630,7 +1658,7 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Imprimación epoxi anticorrosiva de alto contenido en sólidos para saneado de viguetas voladizos</t>
+          <t>Imprimación epoxi anticorrosiva de alto contenido en sólidos para saneado viguetas voladizos</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
@@ -1657,7 +1685,7 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>Materiales y perfiles en ACERO INOXIDABLE (AISI 304/316) para 2 escaleras con crinolina y cancelas</t>
+          <t>Materiales perfiles, peldaños y cancelas en ACERO INOXIDABLE para 2 escalas con crinolina</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
@@ -1679,25 +1707,24 @@
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>MO-01</t>
+          <t>MAT-07</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>Mano de obra especializada montaje HAM obra base (cuadrilla de 4 oficiales ~800 h)</t>
+          <t>Materiales sistema línea de vida LuxTop® (cable AISI 316, postes absorbedores, tensor y carros)</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>horas</t>
+          <t>lote</t>
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>800</v>
-      </c>
-      <c r="E17" s="20">
-        <f>B7</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>10300</v>
       </c>
       <c r="F17" s="20">
         <f>D17*E17</f>
@@ -1707,12 +1734,12 @@
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>MO-02</t>
+          <t>MO-01</t>
         </is>
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>Mano de obra montaje e instalación de 2 escaleras inox con crinolina (~60 h taller y montaje)</t>
+          <t>Mano de obra especializada montaje HAM obra base (cuadrilla de 4 oficiales ~800 h)</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
@@ -1721,7 +1748,7 @@
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>60</v>
+        <v>800</v>
       </c>
       <c r="E18" s="20">
         <f>B7</f>
@@ -1735,24 +1762,25 @@
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>LOG-01</t>
+          <t>MO-02</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Fletes marítimos Península-Menorca para transporte de trailers especiales con paneles de gran formato</t>
+          <t>Mano de obra taller y montaje 2 escalas inox + instalación/ensayo línea LuxTop (~100 h)</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>lote</t>
+          <t>horas</t>
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="20" t="n">
-        <v>5200</v>
+        <v>100</v>
+      </c>
+      <c r="E19" s="20">
+        <f>B7</f>
+        <v/>
       </c>
       <c r="F19" s="20">
         <f>D19*E19</f>
@@ -1762,12 +1790,12 @@
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>LOG-02</t>
+          <t>LOG-01</t>
         </is>
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>Camión grúa pluma autopropulsada para descarga e izado distribuido sobre pórticos en aeropuerto</t>
+          <t>Fletes marítimos Península-Menorca para transporte de trailers especiales paneles gran formato</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
@@ -1779,7 +1807,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>4600</v>
+        <v>5200</v>
       </c>
       <c r="F20" s="20">
         <f>D20*E20</f>
@@ -1789,12 +1817,12 @@
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>LOG-03</t>
+          <t>LOG-02</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>Alquiler de 2 plataformas elevadoras móviles de personal (PEMP) articuladas durante montaje</t>
+          <t>Camión grúa pluma autopropulsada para descarga e izado distribuido sobre pórticos</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -1806,7 +1834,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="20" t="n">
-        <v>3400</v>
+        <v>4600</v>
       </c>
       <c r="F21" s="20">
         <f>D21*E21</f>
@@ -1816,12 +1844,12 @@
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>PRL-01</t>
+          <t>LOG-03</t>
         </is>
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>Protecciones colectivas: redes anticaídas bajo faldones UNE-EN 1263-1 y líneas de vida EN 795</t>
+          <t>Alquiler de 2 plataformas elevadoras móviles de personal (PEMP) articuladas para montaje</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
@@ -1833,7 +1861,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>3800</v>
+        <v>3400</v>
       </c>
       <c r="F22" s="20">
         <f>D22*E22</f>
@@ -1843,12 +1871,12 @@
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>PRL-02</t>
+          <t>PRL-01</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Canon de vertedero insular y tasas de centro de reciclaje autorizado de Menorca</t>
+          <t>Protecciones colectivas: redes anticaídas bajo faldones UNE-EN 1263-1 y líneas de vida EN 795</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
@@ -1860,7 +1888,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="20" t="n">
-        <v>1800</v>
+        <v>3800</v>
       </c>
       <c r="F23" s="20">
         <f>D23*E23</f>
@@ -1868,113 +1896,140 @@
       </c>
     </row>
     <row r="24">
-      <c r="E24" s="43" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>PRL-02</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Canon de vertedero insular y tasas de centro de reciclaje autorizado de Menorca</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F24" s="20">
+        <f>D24*E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" s="43" t="inlineStr">
         <is>
           <t>COSTE DIRECTO TOTAL GLOBAL (CDT HAM):</t>
         </is>
       </c>
-      <c r="F24" s="44">
-        <f>SUM(F11:F23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="F25" s="44">
+        <f>SUM(F11:F24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>CUADRO DE RENTABILIDAD Y BENEFICIO COMERCIAL</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="45" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="45" t="inlineStr">
         <is>
           <t>Concepto Económico</t>
         </is>
       </c>
-      <c r="B27" s="45" t="inlineStr">
+      <c r="B28" s="45" t="inlineStr">
         <is>
           <t>Obra Base (€)</t>
         </is>
       </c>
-      <c r="C27" s="45" t="inlineStr">
-        <is>
-          <t>Opcionales Inox (€)</t>
-        </is>
-      </c>
-      <c r="D27" s="45" t="inlineStr">
+      <c r="C28" s="45" t="inlineStr">
+        <is>
+          <t>Opcionales (€)</t>
+        </is>
+      </c>
+      <c r="D28" s="45" t="inlineStr">
         <is>
           <t>Total Global (€)</t>
         </is>
       </c>
-      <c r="E27" s="45" t="inlineStr">
+      <c r="E28" s="45" t="inlineStr">
         <is>
           <t>% Margen Global</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="46" t="inlineStr">
-        <is>
-          <t>Precio de Venta al Cliente (Base Imp.):</t>
-        </is>
-      </c>
-      <c r="B28" s="47" t="n">
-        <v>220225</v>
-      </c>
-      <c r="C28" s="47" t="n">
-        <v>9800</v>
-      </c>
-      <c r="D28" s="47">
-        <f>B28+C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="48" t="inlineStr">
-        <is>
-          <t>100.00%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="46" t="inlineStr">
         <is>
-          <t>Coste Directo Total HAM:</t>
+          <t>Precio de Venta al Cliente (Base Imp.):</t>
         </is>
       </c>
       <c r="B29" s="47" t="n">
-        <v>125530</v>
+        <v>220225</v>
       </c>
       <c r="C29" s="47" t="n">
-        <v>5380</v>
+        <v>30740</v>
       </c>
       <c r="D29" s="47">
         <f>B29+C29</f>
         <v/>
       </c>
-      <c r="E29" s="48">
-        <f>D29/D28</f>
-        <v/>
+      <c r="E29" s="48" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="49" t="inlineStr">
+      <c r="A30" s="46" t="inlineStr">
+        <is>
+          <t>Coste Directo Total HAM:</t>
+        </is>
+      </c>
+      <c r="B30" s="47" t="n">
+        <v>125530</v>
+      </c>
+      <c r="C30" s="47" t="n">
+        <v>16800</v>
+      </c>
+      <c r="D30" s="47">
+        <f>B30+C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="48">
+        <f>D30/D29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
         <is>
           <t>Margen Bruto de Explotación HAM:</t>
         </is>
       </c>
-      <c r="B30" s="50">
-        <f>B28-B29</f>
-        <v/>
-      </c>
-      <c r="C30" s="50">
-        <f>C28-C29</f>
-        <v/>
-      </c>
-      <c r="D30" s="50">
-        <f>D28-D29</f>
-        <v/>
-      </c>
-      <c r="E30" s="51">
-        <f>D30/D28</f>
+      <c r="B31" s="50">
+        <f>B29-B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="50">
+        <f>C29-C30</f>
+        <v/>
+      </c>
+      <c r="D31" s="50">
+        <f>D29-D30</f>
+        <v/>
+      </c>
+      <c r="E31" s="51">
+        <f>D31/D29</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(presupuestos): actualizar tarifas solicitadas (01 a 25e, 02/03 a 135e, 04 a 95e), integrar medios auxiliares en partidas y desglosar remates partida 05 en P-2026-0044
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
+++ b/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -749,7 +749,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado especial anticorrosión marina Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones bimetálicas inox A2 + EPDM | Opcionales: 2 escalas de gato inox con crinolina (+30%) + Línea de vida permanente LuxTop® (18.000 €)</t>
+          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado Granite® HDX55 (55 µm) por AMBAS CARAS | Medios mecánicos y fletes integrados en partidas principales | Opcionales: 2 escalas de gato inox con crinolina (+30%) + Línea de vida permanente LuxTop® (18.000 €)</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>VALORACIÓN ECONÓMICA DE PARTIDAS BASE</t>
+          <t>VALORACIÓN ECONÓMICA DE PARTIDAS BASE (CON MEDIOS INTEGRADOS)</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       <c r="B20" s="18" t="inlineStr">
         <is>
           <t>Desmontaje controlado de cubierta actual, voladizos existentes y gestión autorizada de residuos
-Desmontaje manual y mecánico de la cubierta y voladizos existentes de chapa/panel degradada y corroída. Descenso a cota cero mediante camión pluma y plataforma elevadora, clasificación de residuos férricos, carga, transporte y entrega en centro autorizado de gestión y reciclaje de residuos de Menorca, incluyendo tasas y canon oficial de vertedero.</t>
+Desmontaje manual y mecánico de la cubierta y voladizos existentes de chapa/panel degradada y corroída. Incluye descenso a cota cero con grúa pluma y plataforma elevadora (medios integrados), acopio, clasificación de residuos férricos, carga, transporte y entrega en centro autorizado de gestión y reciclaje de residuos de Menorca, con tasas y canon oficial de vertedero incluidos.</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
@@ -961,7 +961,7 @@
         <v>1904</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>14.5</v>
+        <v>25</v>
       </c>
       <c r="F20" s="20">
         <f>D20*E20</f>
@@ -977,7 +977,7 @@
       <c r="B21" s="18" t="inlineStr">
         <is>
           <t>Suministro e instalación de Panel Sándwich HDX55 en AMBAS CARAS en cubierta a dos aguas
-Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado, compuesto por núcleo aislante rígido de PIR de 40 mm de espesor (densidad 40 kg/m³, λ = 0,022 W/m·K, clasificación al fuego B-s1,d0) y dos chapas de acero estructural galvanizado con revestimiento de protección marina severa Granite® HDX55 (55 µm de espesor) en AMBAS CARAS (exterior e interior). Fijación a estructura portante mediante tornillería bimetálica autotaladrante de acero inoxidable A2 con arandela estanca de EPDM, con cordón continuo de masilla de butilo en solapes.</t>
+Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado, compuesto por núcleo aislante rígido de PIR de 40 mm de espesor (densidad 40 kg/m³, λ = 0,022 W/m·K, clasificación al fuego B-s1,d0) y dos chapas de acero estructural galvanizado con revestimiento Granite® HDX55 (55 µm de espesor) en AMBAS CARAS (exterior e interior). Fijación a estructura portante mediante tornillería bimetálica autotaladrante de acero inoxidable A2 con arandela estanca de EPDM, con cordón continuo de masilla de butilo en solapes. Incluye fletes marítimos Península-Menorca de paneles de gran longitud, camión grúa pluma para descarga e izado distribuido en pórticos y plataformas elevadoras PEMP integradas.</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -989,7 +989,7 @@
         <v>1042.5</v>
       </c>
       <c r="E21" s="20" t="n">
-        <v>78</v>
+        <v>135</v>
       </c>
       <c r="F21" s="20">
         <f>D21*E21</f>
@@ -1005,7 +1005,7 @@
       <c r="B22" s="18" t="inlineStr">
         <is>
           <t>Suministro e instalación de Panel Sándwich HDX55 en AMBAS CARAS en cubierta a un agua
-Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado (espesor 40 mm PIR, B-s1,d0) con acabado de alta durabilidad Granite® HDX55 (55 µm) por ambas caras (exterior e interior) en faldón a un agua. Incluye adaptaciones mecánicas de faldón, cortes en encuentros contra paramentos verticales y petos, fijaciones inoxidables A2 con arandela de estanqueidad EPDM y sellado butílico continuo.</t>
+Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado (espesor 40 mm PIR, B-s1,d0) con acabado de alta durabilidad Granite® HDX55 (55 µm) por ambas caras (exterior e interior) en faldón a un agua. Incluye adaptaciones mecánicas de faldón, cortes en encuentros contra paramentos verticales y petos, fijaciones inoxidables A2 con arandela de estanqueidad EPDM, sellado butílico continuo y repercusión íntegra de fletes marítimos y medios mecánicos de elevación y PEMP.</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
@@ -1017,7 +1017,7 @@
         <v>328.5</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>80</v>
+        <v>135</v>
       </c>
       <c r="F22" s="20">
         <f>D22*E22</f>
@@ -1033,7 +1033,7 @@
       <c r="B23" s="18" t="inlineStr">
         <is>
           <t>Sustitución integral de voladizos en muelles de carga con acabado HDX55 e imprimación anticorrosiva
-Rehabilitación y sustitución completa de la envolvente de los voladizos de fachada (muelles de carga, 267 m² por fachada, total 533 m²). Incluye cepillado y saneado mecánico superficial con eliminación de óxido en viguetas metálicas en ménsula existentes, aplicación de capa de imprimación epoxi anticorrosiva rica en zinc de alto espesor (C5-M), e instalación de nueva cobertura con chapa/panel de alta resistencia protegida con revestimiento HDX55 (55 µm) en ambas caras, con fijaciones inoxidables A2 y remates perimetrales de goterón frontal.</t>
+Rehabilitación y sustitución completa de la envolvente de los voladizos de fachada (muelles de carga, 267 m² por fachada, total 533 m²). Incluye cepillado y saneado mecánico superficial con eliminación de óxido en viguetas metálicas en ménsula existentes, aplicación de capa de imprimación epoxi anticorrosiva rica en zinc de alto espesor (C5-M), e instalación de nueva cobertura con chapa/panel de alta resistencia protegida con revestimiento HDX55 (55 µm) en ambas caras, con fijaciones inoxidables A2, remates perimetrales frontales con goterón y repercusión de plataformas elevadoras PEMP.</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
@@ -1045,7 +1045,7 @@
         <v>533</v>
       </c>
       <c r="E23" s="20" t="n">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="F23" s="20">
         <f>D23*E23</f>
@@ -1061,7 +1061,7 @@
       <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Rematería completa en acero con acabado HDX55, coronaciones, encuentros, mordidos y sellados
-Suministro, conformación y colocación de toda la rematería técnica necesaria para la total estanqueidad del conjunto, fabricada en chapa de acero galvanizado con idéntico revestimiento HDX55 (55 µm): cumbreras conformadas y troqueladas a dos aguas, remates laterales de testero y coronación de hastiales, baberos de encuentro con paramentos verticales, mordidos mecánicos y adaptación a salidas de ventilación, bajantes, chimeneas y elementos singulares, con sellado perimetral continuo con masilla elástica de poliuretano exterior.</t>
+Suministro, conformación en taller y montaje de 489,15 ml de rematería técnica plegada a medida (desarrollos 300-500 mm) en chapa de acero galvanizado con idéntico recubrimiento Granite® HDX55 (55 µm): 50,23 ml de cumbrera troquelada a dos aguas, 63,34 ml de remates laterales de hastial/testero con goterón, 30,22 ml de babero de coronación contra peto, 10,40 ml de remate de salto entre naves, 174,08 ml de goterones frontales y laterales de voladizo, 160,88 ml de baberos de encuentro voladizo-fachada y 10 unidades de mordidos y cajeados estancos en salidas de chimeneas y bajantes, con doble sellado perimetral continuo con masilla hidro-expansiva de butilo y polímero elástico MS exterior.</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
@@ -1088,8 +1088,8 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>Logística insular, transporte marítimo especial a Menorca y medios pesados de elevación
-Fletes marítimos Península-Menorca para transporte especial de paneles sándwich de gran longitud en trailers específicos, transporte a terminal de carga del Aeropuerto de Menorca, grúa móvil autopropulsada / camión pluma de gran alcance para descarga, elevación e izado directo distribuido sobre pórticos de cubierta, y alquiler de plataformas elevadoras móviles de personal (PEMP) tipo articulada y de tijera durante todas las fases de desmontaje y montaje.</t>
+          <t>Seguridad y salud, protecciones colectivas en altura y protocolo aeroportuario AENA
+Implantación de medidas de seguridad y salud en altura bajo estricta normativa de AENA en terminal de carga: instalación de redes de seguridad anticaídas bajo faldones según norma UNE-EN 1263-1, líneas de vida provisionales homologadas UNE-EN 795, balizamiento perimetral de zonas de acopio y descarga, tramitación de Coordinación de Actividades Empresariales (CAE) en plataforma aeroportuaria, gestión de acreditaciones del personal y recursos preventivos permanentes en obra.</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
@@ -1101,7 +1101,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="20" t="n">
-        <v>15600</v>
+        <v>9800</v>
       </c>
       <c r="F25" s="20">
         <f>D25*E25</f>
@@ -1109,115 +1109,115 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Seguridad y salud, protecciones colectivas en altura y protocolo aeroportuario Aena
-Implantación de medidas de seguridad y salud en altura bajo estricta normativa de Aena en terminal de carga: instalación de redes de seguridad anticaídas bajo faldones según norma UNE-EN 1263-1, líneas de vida provisionales homologadas UNE-EN 795, balizamiento de zonas de acopio y descarga, tramitación de Coordinación de Actividades Empresariales (CAE) en plataforma aeroportuaria, gestión de acreditaciones del personal y recursos preventivos en obra.</t>
-        </is>
-      </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>lote</t>
-        </is>
-      </c>
-      <c r="D26" s="19" t="n">
+      <c r="E26" s="21" t="inlineStr">
+        <is>
+          <t>Subtotal Base Imponible (Obra Base):</t>
+        </is>
+      </c>
+      <c r="F26" s="22">
+        <f>SUM(F20:F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" s="23" t="inlineStr">
+        <is>
+          <t>I.V.A. (21%) Obra Base:</t>
+        </is>
+      </c>
+      <c r="F27" s="24">
+        <f>F26*0.21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL OBRA BASE (IVA incl.):</t>
+        </is>
+      </c>
+      <c r="F28" s="26">
+        <f>F26+F27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>PARTIDAS OPCIONALES INDEPENDIENTES (ACCESOS EN ACERO INOXIDABLE Y LÍNEA LUXTOP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>Partida</t>
+        </is>
+      </c>
+      <c r="B31" s="28" t="inlineStr">
+        <is>
+          <t>Concepto y Descripción Técnica</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>Precio Unitario (€)</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="inlineStr">
+        <is>
+          <t>Importe (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>OPC-01</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>OPCIONAL 1: Escalera de gato con protección dorsal en acero inoxidable para acceso a voladizo (H ≈ 4,20 m)
+Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso seguro desde cota suelo a voladizo (altura aprox. 4,20 m, desarrollo total 5,30 m con desembarco). Incluye montantes verticales de pletina/tubo inox, peldaños antideslizantes estriados de seguridad, jaula de protección dorsal (crinolina) con aros y tirantes longitudinales en pletina inox a partir de 2,20 m, desembarco superior ensanchado con barandillas de salida de 1.100 mm, compuerta batiente de gravedad/muelle con cierre automático, placa de condena inferior anti-intrusión con candado en acero inoxidable para control de acceso aeroportuario AENA, y anclajes químicos estructurales en acero inox A4.</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="20" t="n">
-        <v>9800</v>
-      </c>
-      <c r="F26" s="20">
-        <f>D26*E26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>Subtotal Base Imponible (Obra Base):</t>
-        </is>
-      </c>
-      <c r="F27" s="22">
-        <f>SUM(F20:F26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="E28" s="23" t="inlineStr">
-        <is>
-          <t>I.V.A. (21%) Obra Base:</t>
-        </is>
-      </c>
-      <c r="F28" s="24">
-        <f>F27*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="E29" s="25" t="inlineStr">
-        <is>
-          <t>TOTAL OBRA BASE (IVA incl.):</t>
-        </is>
-      </c>
-      <c r="F29" s="26">
-        <f>F27+F28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>PARTIDAS OPCIONALES INDEPENDIENTES (ACCESOS EN ACERO INOXIDABLE Y LÍNEA DE VIDA LUXTOP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="27" t="inlineStr">
-        <is>
-          <t>Partida</t>
-        </is>
-      </c>
-      <c r="B32" s="28" t="inlineStr">
-        <is>
-          <t>Concepto y Descripción Técnica</t>
-        </is>
-      </c>
-      <c r="C32" s="27" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="D32" s="27" t="inlineStr">
-        <is>
-          <t>Cantidad</t>
-        </is>
-      </c>
-      <c r="E32" s="27" t="inlineStr">
-        <is>
-          <t>Precio Unitario (€)</t>
-        </is>
-      </c>
-      <c r="F32" s="27" t="inlineStr">
-        <is>
-          <t>Importe (€)</t>
-        </is>
+      <c r="E32" s="20" t="n">
+        <v>5005</v>
+      </c>
+      <c r="F32" s="20">
+        <f>D32*E32</f>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>OPC-01</t>
+          <t>OPC-02</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>OPCIONAL 1: Escalera de gato con protección dorsal en acero inoxidable para acceso a voladizo (H ≈ 4,20 m)
-Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso seguro desde cota suelo a voladizo (altura aprox. 4,20 m, desarrollo total 5,30 m con desembarco). Incluye montantes verticales de pletina/tubo inox, peldaños antideslizantes estriados de seguridad, jaula de protección dorsal (crinolina) con aros y tirantes longitudinales en pletina inox a partir de 2,20 m, desembarco superior ensanchado con barandillas de salida de 1.100 mm, compuerta batiente de gravedad/muelle con cierre automático, placa de condena inferior anti-intrusión con candado en acero inoxidable para control de acceso aeroportuario AENA, y anclajes químicos estructurales en acero inox A4.</t>
+          <t>OPCIONAL 2: Escalera de gato con protección dorsal en acero inoxidable para acceso a cubierta (H ≈ 6,80 m)
+Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso técnico y de mantenimiento a la cubierta principal del edificio (altura aprox. 6,80 m, desarrollo total 7,90 m con desembarco). Incluye montantes de acero inox, peldaños antideslizantes mecanizados, jaula dorsal continua (crinolina) en acero inox a partir de 2,50 m de altura, desembarco superior protegido con barandillas de 1.100 mm y rodapié, puerta batiente de salida con resorte de cierre automático de seguridad, portón inferior abatible de bloqueo anti-intrusión con cerradura/candado de seguridad en acero inoxidable, y fijaciones estructurales en acero inoxidable A4.</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
@@ -1229,7 +1229,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="20" t="n">
-        <v>5005</v>
+        <v>7735</v>
       </c>
       <c r="F33" s="20">
         <f>D33*E33</f>
@@ -1239,13 +1239,13 @@
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>OPC-02</t>
+          <t>OPC-03</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>OPCIONAL 2: Escalera de gato con protección dorsal en acero inoxidable para acceso a cubierta (H ≈ 6,80 m)
-Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso técnico y de mantenimiento a la cubierta principal del edificio (altura aprox. 6,80 m, desarrollo total 7,90 m con desembarco). Incluye montantes de acero inox, peldaños antideslizantes mecanizados, jaula dorsal continua (crinolina) en acero inox a partir de 2,50 m de altura, desembarco superior protegido con barandillas de 1.100 mm y rodapié, puerta batiente de salida con resorte de cierre automático de seguridad, portón inferior abatible de bloqueo anti-intrusión con cerradura/candado de seguridad en acero inoxidable, y fijaciones estructurales en acero inoxidable A4.</t>
+          <t>OPCIONAL 3: Línea de vida permanente homologada marca LUXTOP® s/ UNE-EN 795:2012 Tipo C sobre cubierta
+Suministro, replanteo, montaje y certificación oficial de sistema permanente de línea de vida horizontal continua de cable de acero inoxidable AISI 316 (Ø 8 mm) marca LUXTOP®, conforme a las normas UNE-EN 795:2012 Tipo C y CEN/TS 16415 (homologada para trabajo y rescate de hasta 4 operarios simultáneos). Instalación sobre cubierta de panel sándwich mediante postes terminales e intermedios con absorbedor de impacto dinámico patentado LuxTop®, bases de fijación estancas sobreelevadas con juntas de EPDM (evitando cualquier riesgo de filtración o puente térmico), tensor de cable con testigo micrométrico de tensión, pieza curva/esquina si procede, carros deslizadores pasantes transfronterizos sin necesidad de desconexión manual, placa de marcado identificativa CE, ensayos de tracción en obra y dossier de legalización con certificado visado.</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
@@ -1257,7 +1257,7 @@
         <v>1</v>
       </c>
       <c r="E34" s="20" t="n">
-        <v>7735</v>
+        <v>18000</v>
       </c>
       <c r="F34" s="20">
         <f>D34*E34</f>
@@ -1265,149 +1265,121 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>OPC-03</t>
-        </is>
-      </c>
-      <c r="B35" s="18" t="inlineStr">
-        <is>
-          <t>OPCIONAL 3: Línea de vida permanente homologada marca LuxTop® sobre cubierta
-Suministro, replanteo, montaje y certificación oficial de sistema permanente de línea de vida horizontal continua de cable de acero inoxidable AISI 316 (Ø 8 mm) marca LUXTOP®, conforme a las normas UNE-EN 795:2012 Tipo C y CEN/TS 16415 (homologada para trabajo y rescate de hasta 4 operarios simultáneos). Instalación sobre cubierta de panel sándwich mediante postes terminales e intermedios con absorbedor de impacto dinámico patentado LuxTop®, bases de fijación estancas sobreelevadas con juntas de EPDM (evitando cualquier riesgo de filtración o puente térmico), tensor de cable con testigo micrométrico de tensión, pieza curva/esquina si procede, carros deslizadores pasantes transfronterizos sin necesidad de desconexión manual, placa de marcado identificativa CE, ensayos de tracción en obra y dossier de legalización con certificado visado.</t>
-        </is>
-      </c>
-      <c r="C35" s="17" t="inlineStr">
-        <is>
-          <t>ud</t>
-        </is>
-      </c>
-      <c r="D35" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="20" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F35" s="20">
-        <f>D35*E35</f>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>Subtotal Opcionales (Base Imp.):</t>
+        </is>
+      </c>
+      <c r="F35" s="30">
+        <f>SUM(F32:F34)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="E36" s="29" t="inlineStr">
-        <is>
-          <t>Subtotal Opcionales (Base Imp.):</t>
-        </is>
-      </c>
-      <c r="F36" s="30">
-        <f>SUM(F33:F35)</f>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>I.V.A. (21%) Opcionales:</t>
+        </is>
+      </c>
+      <c r="F36" s="24">
+        <f>F35*0.21</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="E37" s="23" t="inlineStr">
-        <is>
-          <t>I.V.A. (21%) Opcionales:</t>
-        </is>
-      </c>
-      <c r="F37" s="24">
-        <f>F36*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="E38" s="31" t="inlineStr">
+      <c r="E37" s="31" t="inlineStr">
         <is>
           <t>TOTAL OPCIONALES (IVA incl.):</t>
         </is>
       </c>
-      <c r="F38" s="32">
-        <f>F36+F37</f>
+      <c r="F37" s="32">
+        <f>F35+F36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL BASE IMPONIBLE CONJUNTA:</t>
+        </is>
+      </c>
+      <c r="F39" s="34">
+        <f>F26+F35</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="E40" s="33" t="inlineStr">
-        <is>
-          <t>TOTAL BASE IMPONIBLE CONJUNTA:</t>
-        </is>
-      </c>
-      <c r="F40" s="34">
-        <f>F27+F36</f>
+      <c r="E40" s="35" t="inlineStr">
+        <is>
+          <t>I.V.A. (21%) Conjunto:</t>
+        </is>
+      </c>
+      <c r="F40" s="36">
+        <f>F39*0.21</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="E41" s="35" t="inlineStr">
-        <is>
-          <t>I.V.A. (21%) Conjunto:</t>
-        </is>
-      </c>
-      <c r="F41" s="36">
-        <f>F40*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="E42" s="37" t="inlineStr">
+      <c r="E41" s="37" t="inlineStr">
         <is>
           <t>TOTAL GENERAL CONTRATO (IVA incl.):</t>
         </is>
       </c>
-      <c r="F42" s="38">
-        <f>F40+F41</f>
-        <v/>
+      <c r="F41" s="38">
+        <f>F39+F40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>CONDICIONES COMERCIALES Y DE EJECUCIÓN</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>CONDICIONES COMERCIALES Y DE EJECUCIÓN</t>
+          <t>• Forma de pago:</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>40% a la formalización (149.057,48 € base), 30% al acopio e inicio montaje (111.793,11 €) y 30% a la recepción final (111.793,11 €). Las partidas opcionales se facturan según aprobación.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>• Forma de pago:</t>
+          <t>• Plazo de ejecución:</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>40% a la formalización (106.588,90 € base), 30% al acopio e inicio montaje (79.941,68 €) y 30% a la recepción final (79.941,67 €). Las partidas opcionales se facturan según aprobación.</t>
+          <t>5 a 7 semanas laborables desde recepción de paneles en Menorca</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>• Plazo de ejecución:</t>
+          <t>• Garantías:</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>5 a 7 semanas laborables desde recepción de paneles en Menorca</t>
+          <t>10 años en recubrimiento Granite® HDX55, en acero inoxidable y en sistema LuxTop®; 5 años en estanqueidad; 2 años en montaje</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>• Garantías:</t>
+          <t>• Validez de oferta:</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>10 años en recubrimiento Granite® HDX55, en acero inoxidable y en sistema LuxTop®; 5 años en estanqueidad; 2 años en montaje</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>• Validez de oferta:</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>30 días naturales desde la fecha de emisión</t>
         </is>
@@ -1445,7 +1417,7 @@
     <row r="2">
       <c r="A2" s="40" t="inlineStr">
         <is>
-          <t>CONFIDENCIAL: USO INTERNO EXCLUSIVO · OBRA BASE + ESCALERAS INOX (+30%) + LÍNEA LUXTOP</t>
+          <t>CONFIDENCIAL: USO INTERNO EXCLUSIVO · TARIFAS ACTUALIZADAS (01: 25€, 02/03: 135€, 04: 95€) · MEDIOS INTEGRADOS</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1576,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Tornillería bimetálica inox A2 con arandelas EPDM, accesorios fijación y masilla de butilo</t>
+          <t>Tornillería bimetálica inox A2 con arandela EPDM, accesorios fijación y masilla de butilo</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
@@ -1974,7 +1946,7 @@
         </is>
       </c>
       <c r="B29" s="47" t="n">
-        <v>220225</v>
+        <v>307970</v>
       </c>
       <c r="C29" s="47" t="n">
         <v>30740</v>

</xml_diff>

<commit_message>
feat(P-2026-0044): actualizar fijaciones roscachapa galvanizadas, pago a convenir y plazo 2 a 3 meses
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
+++ b/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto.xlsx
@@ -749,7 +749,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado Granite® HDX55 (55 µm) por AMBAS CARAS | Medios mecánicos y fletes integrados en partidas principales | Opcionales: 2 escalas de gato inox con crinolina (+30%) + Línea de vida permanente LuxTop® (18.000 €)</t>
+          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones roscachapa galvanizadas con arandela vulcanizada EPDM | Medios mecánicos y fletes integrados | Opcionales: 2 escalas de gato inox con crinolina (+30%) + Línea LuxTop® (18.000 €)</t>
         </is>
       </c>
     </row>
@@ -977,7 +977,7 @@
       <c r="B21" s="18" t="inlineStr">
         <is>
           <t>Suministro e instalación de Panel Sándwich HDX55 en AMBAS CARAS en cubierta a dos aguas
-Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado, compuesto por núcleo aislante rígido de PIR de 40 mm de espesor (densidad 40 kg/m³, λ = 0,022 W/m·K, clasificación al fuego B-s1,d0) y dos chapas de acero estructural galvanizado con revestimiento Granite® HDX55 (55 µm de espesor) en AMBAS CARAS (exterior e interior). Fijación a estructura portante mediante tornillería bimetálica autotaladrante de acero inoxidable A2 con arandela estanca de EPDM, con cordón continuo de masilla de butilo en solapes. Incluye fletes marítimos Península-Menorca de paneles de gran longitud, camión grúa pluma para descarga e izado distribuido en pórticos y plataformas elevadoras PEMP integradas.</t>
+Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado, compuesto por núcleo aislante rígido de PIR de 40 mm de espesor (densidad 40 kg/m³, λ = 0,022 W/m·K, clasificación al fuego B-s1,d0) y dos chapas de acero estructural galvanizado con revestimiento de protección marina severa Granite® HDX55 (55 µm de espesor) en AMBAS CARAS (exterior e interior). Fijación a estructura portante mediante tornillería roscachapa / autorroscante de acero galvanizado con arandela estanca vulcanizada de EPDM y cordón continuo de masilla hidro-expansiva de butilo en solapes. Incluye fletes marítimos Península-Menorca de paneles de gran longitud, camión grúa pluma para descarga e izado distribuido en pórticos y plataformas elevadoras PEMP integradas.</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -1005,7 +1005,7 @@
       <c r="B22" s="18" t="inlineStr">
         <is>
           <t>Suministro e instalación de Panel Sándwich HDX55 en AMBAS CARAS en cubierta a un agua
-Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado (espesor 40 mm PIR, B-s1,d0) con acabado de alta durabilidad Granite® HDX55 (55 µm) por ambas caras (exterior e interior) en faldón a un agua. Incluye adaptaciones mecánicas de faldón, cortes en encuentros contra paramentos verticales y petos, fijaciones inoxidables A2 con arandela de estanqueidad EPDM, sellado butílico continuo y repercusión íntegra de fletes marítimos y medios mecánicos de elevación y PEMP.</t>
+Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado (espesor 40 mm PIR, B-s1,d0) con acabado de alta durabilidad Granite® HDX55 (55 µm) por ambas caras (exterior e interior) en faldón a un agua. Incluye adaptaciones mecánicas de faldón, cortes en encuentros contra paramentos verticales y petos, fijaciones roscachapa de acero galvanizado con arandela de estanqueidad EPDM, sellado butílico continuo y repercusión íntegra de fletes marítimos y medios mecánicos de elevación y PEMP.</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
@@ -1033,7 +1033,7 @@
       <c r="B23" s="18" t="inlineStr">
         <is>
           <t>Sustitución integral de voladizos en muelles de carga con acabado HDX55 e imprimación anticorrosiva
-Rehabilitación y sustitución completa de la envolvente de los voladizos de fachada (muelles de carga, 267 m² por fachada, total 533 m²). Incluye cepillado y saneado mecánico superficial con eliminación de óxido en viguetas metálicas en ménsula existentes, aplicación de capa de imprimación epoxi anticorrosiva rica en zinc de alto espesor (C5-M), e instalación de nueva cobertura con chapa/panel de alta resistencia protegida con revestimiento HDX55 (55 µm) en ambas caras, con fijaciones inoxidables A2, remates perimetrales frontales con goterón y repercusión de plataformas elevadoras PEMP.</t>
+Rehabilitación y sustitución completa de la envolvente de los voladizos de fachada (muelles de carga, 267 m² por fachada, total 533 m²). Incluye cepillado y saneado mecánico superficial con eliminación de óxido en viguetas metálicas en ménsula existentes, aplicación de capa de imprimación epoxi anticorrosiva rica en zinc de alto espesor (C5-M), e instalación de nueva cobertura con chapa/panel de alta resistencia protegida con revestimiento HDX55 (55 µm) en ambas caras, con tornillería roscachapa galvanizada con arandela EPDM, remates perimetrales frontales con goterón y repercusión de plataformas elevadoras PEMP.</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
@@ -1061,7 +1061,7 @@
       <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Rematería completa en acero con acabado HDX55, coronaciones, encuentros, mordidos y sellados
-Suministro, conformación en taller y montaje de 489,15 ml de rematería técnica plegada a medida (desarrollos 300-500 mm) en chapa de acero galvanizado con idéntico recubrimiento Granite® HDX55 (55 µm): 50,23 ml de cumbrera troquelada a dos aguas, 63,34 ml de remates laterales de hastial/testero con goterón, 30,22 ml de babero de coronación contra peto, 10,40 ml de remate de salto entre naves, 174,08 ml de goterones frontales y laterales de voladizo, 160,88 ml de baberos de encuentro voladizo-fachada y 10 unidades de mordidos y cajeados estancos en salidas de chimeneas y bajantes, con doble sellado perimetral continuo con masilla hidro-expansiva de butilo y polímero elástico MS exterior.</t>
+Suministro, conformación en taller y montaje de 489,15 ml de rematería técnica plegada a medida (desarrollos 300-500 mm) en chapa de acero galvanizado con idéntico recubrimiento Granite® HDX55 (55 µm): 50,23 ml de cumbrera troquelada a dos aguas, 63,34 ml de remates laterales de hastial/testero con goterón, 30,22 ml de babero de coronación contra peto, 10,40 ml de remate de salto entre naves, 174,08 ml de goterones frontales y laterales de voladizo, 160,88 ml de baberos de encuentro voladizo-fachada y 10 unidades de mordidos y cajeados estancos en salidas de chimeneas y bajantes, fijados con tornillería galvanizada lacada con junta EPDM y doble sellado perimetral continuo con masilla hidro-expansiva de butilo y polímero elástico MS exterior.</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>40% a la formalización (149.057,48 € base), 30% al acopio e inicio montaje (111.793,11 €) y 30% a la recepción final (111.793,11 €). Las partidas opcionales se facturan según aprobación.</t>
+          <t>A convenir con el cliente según avance y certificaciones de obra.</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>5 a 7 semanas laborables desde recepción de paneles en Menorca</t>
+          <t>2 a 3 meses desde la recepción de materiales en obra y formalización del contrato.</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Tornillería bimetálica inox A2 con arandela EPDM, accesorios fijación y masilla de butilo</t>
+          <t>Tornillería roscachapa de acero galvanizado con arandela EPDM, accesorios fijación y masilla butilo</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
@@ -1588,7 +1588,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="20" t="n">
-        <v>6200</v>
+        <v>5200</v>
       </c>
       <c r="F13" s="20">
         <f>D13*E13</f>
@@ -1968,7 +1968,7 @@
         </is>
       </c>
       <c r="B30" s="47" t="n">
-        <v>125530</v>
+        <v>124530</v>
       </c>
       <c r="C30" s="47" t="n">
         <v>16800</v>

</xml_diff>